<commit_message>
Jalankan ulang notebook penuh dan tambahkan perhitungan manual per tahap
- Notebook dieksekusi ulang dari Tahap 0 sampai 14 tanpa error (86 sel);
  seluruh output sel kini sinkron dengan kode builder.
- outputs/perhitungan_manual/ berisi 23 berkas tahap_TT_SS_*.md dan
  README.md (daftar isi), dengan tautan sebelumnya/berikutnya di tiap berkas.
- Semua metrik (RMSE, MAE, MAPE, akurasi arah, uji DM) identik dengan run
  sebelumnya; hanya kolom waktu latih (detik) di Tabel 9, 11, 13, 14, 17
  yang berubah karena bergantung pada kecepatan mesin.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WtB1QbCUFRKnrWDJL7ukHK
</commit_message>
<xml_diff>
--- a/outputs/tabel/tabel_09_hasil_tuning_hyperparameter_model_lstm.xlsx
+++ b/outputs/tabel/tabel_09_hasil_tuning_hyperparameter_model_lstm.xlsx
@@ -490,10 +490,10 @@
         <v>7.394564349448522</v>
       </c>
       <c r="G2" t="n">
-        <v>15.45730587399999</v>
+        <v>28.52421552799979</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1545730587399999</v>
+        <v>0.2852421552799979</v>
       </c>
       <c r="I2" t="n">
         <v>851</v>
@@ -522,10 +522,10 @@
         <v>4.819835210396409</v>
       </c>
       <c r="G3" t="n">
-        <v>71.77969295399998</v>
+        <v>131.880415133</v>
       </c>
       <c r="H3" t="n">
-        <v>0.143559385908</v>
+        <v>0.2637608302660001</v>
       </c>
       <c r="I3" t="n">
         <v>851</v>
@@ -554,10 +554,10 @@
         <v>2.787158067460322</v>
       </c>
       <c r="G4" t="n">
-        <v>144.3139483780001</v>
+        <v>255.6384160930002</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1443139483780001</v>
+        <v>0.2556384160930001</v>
       </c>
       <c r="I4" t="n">
         <v>851</v>
@@ -586,10 +586,10 @@
         <v>2.786171857233439</v>
       </c>
       <c r="G5" t="n">
-        <v>17.0124225290001</v>
+        <v>25.12245218999988</v>
       </c>
       <c r="H5" t="n">
-        <v>0.170124225290001</v>
+        <v>0.2512245218999988</v>
       </c>
       <c r="I5" t="n">
         <v>2501</v>
@@ -618,10 +618,10 @@
         <v>2.850487422515137</v>
       </c>
       <c r="G6" t="n">
-        <v>75.60707250599989</v>
+        <v>126.7081228350003</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1512141450119998</v>
+        <v>0.2534162456700005</v>
       </c>
       <c r="I6" t="n">
         <v>2501</v>
@@ -650,10 +650,10 @@
         <v>2.275284708105242</v>
       </c>
       <c r="G7" t="n">
-        <v>148.9218543390002</v>
+        <v>266.9591869870001</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1489218543390002</v>
+        <v>0.2669591869870001</v>
       </c>
       <c r="I7" t="n">
         <v>2501</v>
@@ -682,10 +682,10 @@
         <v>3.418143505239934</v>
       </c>
       <c r="G8" t="n">
-        <v>15.70729154500032</v>
+        <v>30.95125313900007</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1570729154500032</v>
+        <v>0.3095125313900007</v>
       </c>
       <c r="I8" t="n">
         <v>4951</v>
@@ -714,10 +714,10 @@
         <v>2.756503944357636</v>
       </c>
       <c r="G9" t="n">
-        <v>75.13455342299994</v>
+        <v>136.4454199530001</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1502691068459999</v>
+        <v>0.2728908399060001</v>
       </c>
       <c r="I9" t="n">
         <v>4951</v>
@@ -746,10 +746,10 @@
         <v>2.367278641285638</v>
       </c>
       <c r="G10" t="n">
-        <v>149.0980687330002</v>
+        <v>270.9533647829999</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1490980687330002</v>
+        <v>0.2709533647829999</v>
       </c>
       <c r="I10" t="n">
         <v>4951</v>
@@ -778,10 +778,10 @@
         <v>3.012826567149487</v>
       </c>
       <c r="G11" t="n">
-        <v>16.13968675000024</v>
+        <v>29.38009440400037</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1613968675000024</v>
+        <v>0.2938009440400037</v>
       </c>
       <c r="I11" t="n">
         <v>8201</v>
@@ -810,10 +810,10 @@
         <v>1.902486020390829</v>
       </c>
       <c r="G12" t="n">
-        <v>79.56232019599975</v>
+        <v>143.7189331830004</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1591246403919995</v>
+        <v>0.2874378663660009</v>
       </c>
       <c r="I12" t="n">
         <v>8201</v>
@@ -846,10 +846,10 @@
         <v>2.130108430925327</v>
       </c>
       <c r="G13" t="n">
-        <v>154.1919103519999</v>
+        <v>275.9125214039996</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1541919103519999</v>
+        <v>0.2759125214039996</v>
       </c>
       <c r="I13" t="n">
         <v>8201</v>
@@ -878,10 +878,10 @@
         <v>4.972077798803737</v>
       </c>
       <c r="G14" t="n">
-        <v>17.72137000299972</v>
+        <v>29.82708778399956</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1772137000299972</v>
+        <v>0.2982708778399956</v>
       </c>
       <c r="I14" t="n">
         <v>12251</v>
@@ -910,10 +910,10 @@
         <v>3.634662783691574</v>
       </c>
       <c r="G15" t="n">
-        <v>81.1901188060001</v>
+        <v>144.2230929990001</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1623802376120002</v>
+        <v>0.2884461859980001</v>
       </c>
       <c r="I15" t="n">
         <v>12251</v>
@@ -942,10 +942,10 @@
         <v>2.729645926814857</v>
       </c>
       <c r="G16" t="n">
-        <v>155.3721391029999</v>
+        <v>301.0828070739999</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1553721391029999</v>
+        <v>0.3010828070739999</v>
       </c>
       <c r="I16" t="n">
         <v>12251</v>

</xml_diff>